<commit_message>
update low N file (forgot to save)
</commit_message>
<xml_diff>
--- a/hoagland_recipes/NxPxI_hoagland_lowN.xlsx
+++ b/hoagland_recipes/NxPxI_hoagland_lowN.xlsx
@@ -21,7 +21,7 @@
     <sheet name="0 ppm N, 62 ppm P" sheetId="8" r:id="rId6"/>
     <sheet name="0 ppm N, 93 ppm P" sheetId="9" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1252,28 +1252,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">

</xml_diff>